<commit_message>
Added dimension-descriptors in json
</commit_message>
<xml_diff>
--- a/frontend/Backend/excel/Daten.xlsx
+++ b/frontend/Backend/excel/Daten.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Dimensionen_Handlungsfeld_Indik" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Handlungsempfehlung_Indikator_H" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Frage_Handlungsfeld_Antwort_Ind" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Dimension_Beschreibung" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2874" uniqueCount="1316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2884" uniqueCount="1321">
   <si>
     <t xml:space="preserve">ID Dimension</t>
   </si>
@@ -4000,6 +4001,21 @@
   </si>
   <si>
     <t xml:space="preserve">A251</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beschreibung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 4</t>
   </si>
 </sst>
 </file>
@@ -15555,4 +15571,63 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;KffffffSeite &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1316</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>1317</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>1318</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>1319</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>1320</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;KffffffSeite &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>